<commit_message>
Enabled multiple tabs in the OCP pipeline
</commit_message>
<xml_diff>
--- a/outputs/OCP_2_#1.xlsx
+++ b/outputs/OCP_2_#1.xlsx
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Técnica</t>
+          <t>TÃ©cnica</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -490,7 +490,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Duración</t>
+          <t>DuraciÃ³n</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">

</xml_diff>